<commit_message>
registry condition line list
</commit_message>
<xml_diff>
--- a/report_translations.xlsx
+++ b/report_translations.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/salmanraza/Documents/GitHub/tamanu-source-dbt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E1E85D-4D9C-A148-9368-4CA60E1B1E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03729B65-B003-9F4D-A372-25B3E9C119B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1160" yWindow="980" windowWidth="27640" windowHeight="15440" xr2:uid="{FB1CF5DC-2DD9-EF4F-98DC-2283187EABD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Translated String" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Translated String'!$A$1:$B$1</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="517">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="529">
   <si>
     <t>stringId</t>
   </si>
@@ -1587,6 +1590,42 @@
   </si>
   <si>
     <t>Schedule</t>
+  </si>
+  <si>
+    <t>Condition added by</t>
+  </si>
+  <si>
+    <t>report.reporting.registryRegistrationStatus</t>
+  </si>
+  <si>
+    <t>Registry Status</t>
+  </si>
+  <si>
+    <t>report.reporting.patientDivision</t>
+  </si>
+  <si>
+    <t>report.reporting.patientSubDivision</t>
+  </si>
+  <si>
+    <t>report.reporting.patientMedicalArea</t>
+  </si>
+  <si>
+    <t>Medical Area</t>
+  </si>
+  <si>
+    <t>Sub Division</t>
+  </si>
+  <si>
+    <t>Division</t>
+  </si>
+  <si>
+    <t>report.reporting.registryConditionRecordedBy</t>
+  </si>
+  <si>
+    <t>report.reporting.registryConditionRecordedDate</t>
+  </si>
+  <si>
+    <t>Date condition added</t>
   </si>
 </sst>
 </file>
@@ -1958,8 +1997,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D06625-878C-A840-A829-5EB8C3969019}">
-  <dimension ref="A1:B268"/>
+  <dimension ref="A1:B274"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="39.33203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -2643,50 +2686,50 @@
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="B86" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B87" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B88" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B89" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B90" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B91" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
@@ -2979,18 +3022,18 @@
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B128" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B129" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.2">
@@ -3611,501 +3654,554 @@
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B207" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B208" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="B209" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
-        <v>402</v>
+        <v>520</v>
       </c>
       <c r="B210" t="s">
-        <v>403</v>
+        <v>525</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
-        <v>404</v>
+        <v>521</v>
       </c>
       <c r="B211" t="s">
-        <v>405</v>
+        <v>524</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
-        <v>406</v>
+        <v>522</v>
       </c>
       <c r="B212" t="s">
-        <v>407</v>
+        <v>523</v>
       </c>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
       <c r="B213" t="s">
-        <v>409</v>
+        <v>403</v>
       </c>
     </row>
     <row r="214" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
-        <v>410</v>
+        <v>404</v>
       </c>
       <c r="B214" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="B215" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
-        <v>414</v>
+        <v>408</v>
       </c>
       <c r="B216" t="s">
-        <v>415</v>
+        <v>409</v>
       </c>
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
-        <v>416</v>
+        <v>410</v>
       </c>
       <c r="B217" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
       <c r="B218" t="s">
-        <v>419</v>
+        <v>413</v>
       </c>
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
-        <v>420</v>
+        <v>414</v>
       </c>
       <c r="B219" t="s">
-        <v>421</v>
+        <v>415</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="B220" t="s">
-        <v>423</v>
+        <v>417</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
       <c r="B221" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
       <c r="B222" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
       <c r="B223" t="s">
-        <v>429</v>
+        <v>423</v>
       </c>
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="B224" t="s">
-        <v>431</v>
+        <v>425</v>
       </c>
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
-        <v>432</v>
+        <v>426</v>
       </c>
       <c r="B225" t="s">
-        <v>433</v>
+        <v>427</v>
       </c>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="B226" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="B227" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="B228" t="s">
-        <v>439</v>
+        <v>433</v>
       </c>
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
-        <v>440</v>
+        <v>434</v>
       </c>
       <c r="B229" t="s">
-        <v>441</v>
+        <v>435</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
       <c r="B230" t="s">
-        <v>443</v>
+        <v>437</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
       <c r="B231" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
       <c r="B232" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="B233" t="s">
-        <v>237</v>
+        <v>443</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="B234" t="s">
-        <v>450</v>
+        <v>445</v>
       </c>
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
-        <v>451</v>
+        <v>446</v>
       </c>
       <c r="B235" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
       <c r="B236" t="s">
-        <v>454</v>
+        <v>237</v>
       </c>
     </row>
     <row r="237" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
-        <v>455</v>
+        <v>526</v>
       </c>
       <c r="B237" t="s">
-        <v>47</v>
+        <v>517</v>
       </c>
     </row>
     <row r="238" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
-        <v>456</v>
+        <v>527</v>
       </c>
       <c r="B238" t="s">
-        <v>457</v>
+        <v>528</v>
       </c>
     </row>
     <row r="239" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="B239" t="s">
-        <v>459</v>
+        <v>452</v>
       </c>
     </row>
     <row r="240" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
-        <v>460</v>
+        <v>449</v>
       </c>
       <c r="B240" t="s">
-        <v>461</v>
+        <v>450</v>
       </c>
     </row>
     <row r="241" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
-        <v>462</v>
+        <v>453</v>
       </c>
       <c r="B241" t="s">
-        <v>463</v>
+        <v>454</v>
       </c>
     </row>
     <row r="242" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="B242" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
     </row>
     <row r="243" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="B243" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
-        <v>468</v>
+        <v>455</v>
       </c>
       <c r="B244" t="s">
-        <v>273</v>
+        <v>47</v>
       </c>
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
-        <v>469</v>
+        <v>456</v>
       </c>
       <c r="B245" t="s">
-        <v>470</v>
+        <v>457</v>
       </c>
     </row>
     <row r="246" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
-        <v>471</v>
+        <v>458</v>
       </c>
       <c r="B246" t="s">
-        <v>472</v>
+        <v>459</v>
       </c>
     </row>
     <row r="247" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
-        <v>473</v>
+        <v>518</v>
       </c>
       <c r="B247" t="s">
-        <v>474</v>
+        <v>519</v>
       </c>
     </row>
     <row r="248" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
-        <v>475</v>
+        <v>464</v>
       </c>
       <c r="B248" t="s">
-        <v>476</v>
+        <v>465</v>
       </c>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
-        <v>477</v>
+        <v>466</v>
       </c>
       <c r="B249" t="s">
-        <v>478</v>
+        <v>467</v>
       </c>
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
-        <v>479</v>
+        <v>468</v>
       </c>
       <c r="B250" t="s">
-        <v>480</v>
+        <v>273</v>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
-        <v>481</v>
+        <v>469</v>
       </c>
       <c r="B251" t="s">
-        <v>482</v>
+        <v>470</v>
       </c>
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
-        <v>483</v>
+        <v>471</v>
       </c>
       <c r="B252" t="s">
-        <v>484</v>
+        <v>472</v>
       </c>
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
-        <v>485</v>
+        <v>473</v>
       </c>
       <c r="B253" t="s">
-        <v>486</v>
+        <v>474</v>
       </c>
     </row>
     <row r="254" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
-        <v>487</v>
+        <v>475</v>
       </c>
       <c r="B254" t="s">
-        <v>488</v>
+        <v>476</v>
       </c>
     </row>
     <row r="255" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
-        <v>489</v>
+        <v>477</v>
       </c>
       <c r="B255" t="s">
-        <v>490</v>
+        <v>478</v>
       </c>
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="B256" t="s">
-        <v>492</v>
+        <v>480</v>
       </c>
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
-        <v>493</v>
+        <v>481</v>
       </c>
       <c r="B257" t="s">
-        <v>494</v>
+        <v>482</v>
       </c>
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
-        <v>495</v>
+        <v>483</v>
       </c>
       <c r="B258" t="s">
-        <v>496</v>
+        <v>484</v>
       </c>
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
-        <v>497</v>
+        <v>485</v>
       </c>
       <c r="B259" t="s">
-        <v>498</v>
+        <v>486</v>
       </c>
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A260" t="s">
-        <v>499</v>
+        <v>487</v>
       </c>
       <c r="B260" t="s">
-        <v>500</v>
+        <v>488</v>
       </c>
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A261" t="s">
-        <v>501</v>
+        <v>489</v>
       </c>
       <c r="B261" t="s">
-        <v>502</v>
+        <v>490</v>
       </c>
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A262" t="s">
-        <v>503</v>
+        <v>491</v>
       </c>
       <c r="B262" t="s">
-        <v>504</v>
+        <v>492</v>
       </c>
     </row>
     <row r="263" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A263" t="s">
-        <v>505</v>
+        <v>493</v>
       </c>
       <c r="B263" t="s">
-        <v>506</v>
+        <v>494</v>
       </c>
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A264" t="s">
-        <v>507</v>
+        <v>495</v>
       </c>
       <c r="B264" t="s">
-        <v>508</v>
+        <v>496</v>
       </c>
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A265" t="s">
-        <v>509</v>
+        <v>497</v>
       </c>
       <c r="B265" t="s">
-        <v>510</v>
+        <v>498</v>
       </c>
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A266" t="s">
-        <v>511</v>
+        <v>499</v>
       </c>
       <c r="B266" t="s">
-        <v>512</v>
+        <v>500</v>
       </c>
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A267" t="s">
-        <v>513</v>
+        <v>501</v>
       </c>
       <c r="B267" t="s">
-        <v>514</v>
+        <v>502</v>
       </c>
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A268" t="s">
+        <v>503</v>
+      </c>
+      <c r="B268" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A269" t="s">
+        <v>505</v>
+      </c>
+      <c r="B269" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A270" t="s">
+        <v>507</v>
+      </c>
+      <c r="B270" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A271" t="s">
+        <v>509</v>
+      </c>
+      <c r="B271" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A272" t="s">
+        <v>511</v>
+      </c>
+      <c r="B272" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A273" t="s">
+        <v>513</v>
+      </c>
+      <c r="B273" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A274" t="s">
         <v>515</v>
       </c>
-      <c r="B268" t="s">
+      <c r="B274" t="s">
         <v>516</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B1" xr:uid="{57D06625-878C-A840-A829-5EB8C3969019}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B271">
+      <sortCondition ref="A1:A271"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
MAUI-5498: Encounter Diet Line List (#194)
</commit_message>
<xml_diff>
--- a/report_translations.xlsx
+++ b/report_translations.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/salmanraza/Documents/GitHub/tamanu-source-dbt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E1E85D-4D9C-A148-9368-4CA60E1B1E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C2643C9-F5FA-BC43-A9F0-6DB72EAF824A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1160" yWindow="980" windowWidth="27640" windowHeight="15440" xr2:uid="{FB1CF5DC-2DD9-EF4F-98DC-2283187EABD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Translated String" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Translated String'!$A$1:$B$1</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="517">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="519">
   <si>
     <t>stringId</t>
   </si>
@@ -1587,6 +1590,12 @@
   </si>
   <si>
     <t>Schedule</t>
+  </si>
+  <si>
+    <t>report.reporting.patientAllergies</t>
+  </si>
+  <si>
+    <t>Allergies</t>
   </si>
 </sst>
 </file>
@@ -1958,8 +1967,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D06625-878C-A840-A829-5EB8C3969019}">
-  <dimension ref="A1:B268"/>
+  <dimension ref="A1:B269"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="38.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -2643,50 +2655,50 @@
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="B86" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B87" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B88" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B89" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B90" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B91" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
@@ -2979,18 +2991,18 @@
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B128" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B129" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.2">
@@ -3363,258 +3375,258 @@
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
-        <v>336</v>
+        <v>517</v>
       </c>
       <c r="B176" t="s">
-        <v>337</v>
+        <v>518</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B177" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B178" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B179" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B180" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B181" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B182" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="B183" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B184" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B185" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B186" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B187" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B188" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B189" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B190" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B191" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B192" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B193" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B194" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B195" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B196" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B197" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B198" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B199" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B200" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B201" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B202" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="203" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B203" t="s">
-        <v>47</v>
+        <v>389</v>
       </c>
     </row>
     <row r="204" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B204" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="205" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B205" t="s">
-        <v>393</v>
+        <v>49</v>
       </c>
     </row>
     <row r="206" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B206" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B207" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.2">
@@ -3635,202 +3647,202 @@
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
       <c r="B210" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B211" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B212" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B213" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="214" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B214" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B215" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B216" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B217" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="B218" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="B219" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B220" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B221" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B222" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="B223" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B224" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B225" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="B226" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B227" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B228" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="B229" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B230" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B231" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="B232" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="B233" t="s">
-        <v>237</v>
+        <v>447</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B234" t="s">
-        <v>450</v>
+        <v>237</v>
       </c>
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.2">
@@ -3843,269 +3855,282 @@
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="B236" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
     </row>
     <row r="237" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="B237" t="s">
-        <v>47</v>
+        <v>454</v>
       </c>
     </row>
     <row r="238" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="B238" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
     </row>
     <row r="239" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="B239" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
     </row>
     <row r="240" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
-        <v>460</v>
+        <v>455</v>
       </c>
       <c r="B240" t="s">
-        <v>461</v>
+        <v>47</v>
       </c>
     </row>
     <row r="241" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
-        <v>462</v>
+        <v>456</v>
       </c>
       <c r="B241" t="s">
-        <v>463</v>
+        <v>457</v>
       </c>
     </row>
     <row r="242" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
-        <v>464</v>
+        <v>458</v>
       </c>
       <c r="B242" t="s">
-        <v>465</v>
+        <v>459</v>
       </c>
     </row>
     <row r="243" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="B243" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="B244" t="s">
-        <v>273</v>
+        <v>467</v>
       </c>
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B245" t="s">
-        <v>470</v>
+        <v>273</v>
       </c>
     </row>
     <row r="246" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="B246" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="247" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="B247" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="248" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="B248" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B249" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="B250" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="B251" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="B252" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="B253" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="254" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B254" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="255" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="B255" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="B256" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="B257" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="B258" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="B259" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A260" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="B260" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A261" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="B261" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A262" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B262" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="263" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A263" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B263" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A264" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B264" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A265" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="B265" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A266" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="B266" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A267" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="B267" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A268" t="s">
+        <v>513</v>
+      </c>
+      <c r="B268" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A269" t="s">
         <v>515</v>
       </c>
-      <c r="B268" t="s">
+      <c r="B269" t="s">
         <v>516</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B1" xr:uid="{57D06625-878C-A840-A829-5EB8C3969019}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B269">
+      <sortCondition ref="A1:A269"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
MAUI-5498: Encounter Diet Line List [Tiny] (#196)
</commit_message>
<xml_diff>
--- a/report_translations.xlsx
+++ b/report_translations.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/salmanraza/Documents/GitHub/tamanu-source-dbt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C2643C9-F5FA-BC43-A9F0-6DB72EAF824A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70BED706-15E6-EA43-94C4-45829D5E8A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1160" yWindow="980" windowWidth="27640" windowHeight="15440" xr2:uid="{FB1CF5DC-2DD9-EF4F-98DC-2283187EABD8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="523">
   <si>
     <t>stringId</t>
   </si>
@@ -1596,6 +1596,18 @@
   </si>
   <si>
     <t>Allergies</t>
+  </si>
+  <si>
+    <t>report.reporting.encounterStartDate</t>
+  </si>
+  <si>
+    <t>report.reporting.encounterStartTime</t>
+  </si>
+  <si>
+    <t>Encounter start time</t>
+  </si>
+  <si>
+    <t>Encounter start date</t>
   </si>
 </sst>
 </file>
@@ -1967,10 +1979,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D06625-878C-A840-A829-5EB8C3969019}">
-  <dimension ref="A1:B269"/>
+  <dimension ref="A1:B271"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="38.1640625" customWidth="1"/>
+    <col min="1" max="1" width="58.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -2719,1416 +2731,1432 @@
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>182</v>
+        <v>519</v>
       </c>
       <c r="B94" t="s">
-        <v>183</v>
+        <v>522</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B95" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>186</v>
+        <v>520</v>
       </c>
       <c r="B96" t="s">
-        <v>187</v>
+        <v>521</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B97" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B98" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B99" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B100" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B101" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B102" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="B103" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B104" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B105" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B106" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B107" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B108" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B109" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="B110" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="B111" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="B112" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B113" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="B114" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B115" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="B116" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B117" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="B118" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="B119" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="B120" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="B121" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="B122" t="s">
-        <v>185</v>
+        <v>235</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="B123" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B124" t="s">
-        <v>242</v>
+        <v>185</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="B125" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="B126" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="B127" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="B128" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B129" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B130" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="B131" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="B132" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="B133" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="B134" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="B135" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="B136" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="B137" t="s">
-        <v>219</v>
+        <v>264</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="B138" t="s">
-        <v>233</v>
+        <v>266</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B139" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B140" t="s">
-        <v>271</v>
+        <v>233</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B141" t="s">
-        <v>273</v>
+        <v>221</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="B142" t="s">
-        <v>231</v>
+        <v>271</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="B143" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B144" t="s">
-        <v>277</v>
+        <v>231</v>
       </c>
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B145" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="B146" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="B147" t="s">
-        <v>282</v>
+        <v>227</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="B148" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="B149" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="B150" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B151" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="B152" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="B153" t="s">
-        <v>237</v>
+        <v>290</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="B154" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="B155" t="s">
-        <v>297</v>
+        <v>237</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="B156" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="B157" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="B158" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="B159" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="B160" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="B161" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="B162" t="s">
-        <v>62</v>
+        <v>307</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="B163" t="s">
-        <v>19</v>
+        <v>309</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B164" t="s">
-        <v>313</v>
+        <v>62</v>
       </c>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="B165" t="s">
-        <v>315</v>
+        <v>19</v>
       </c>
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="B166" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="B167" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="B168" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="B169" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B170" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="B171" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="B172" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="B173" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="B174" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="B175" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
-        <v>517</v>
+        <v>332</v>
       </c>
       <c r="B176" t="s">
-        <v>518</v>
+        <v>333</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B177" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
-        <v>338</v>
+        <v>517</v>
       </c>
       <c r="B178" t="s">
-        <v>339</v>
+        <v>518</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="B179" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="B180" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="B181" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="B182" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="B183" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="B184" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="B185" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="B186" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="B187" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="B188" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="B189" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="B190" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="B191" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="B192" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="B193" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="B194" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="B195" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="B196" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="B197" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="B198" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="B199" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="B200" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="B201" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="B202" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
     </row>
     <row r="203" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="B203" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
     </row>
     <row r="204" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="B204" t="s">
-        <v>47</v>
+        <v>387</v>
       </c>
     </row>
     <row r="205" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="B205" t="s">
-        <v>49</v>
+        <v>389</v>
       </c>
     </row>
     <row r="206" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B206" t="s">
-        <v>393</v>
+        <v>47</v>
       </c>
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="B207" t="s">
-        <v>395</v>
+        <v>49</v>
       </c>
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="B208" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="B209" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B210" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B211" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
-        <v>404</v>
+        <v>396</v>
       </c>
       <c r="B212" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="B213" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
     </row>
     <row r="214" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="B214" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="B215" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="B216" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
       <c r="B217" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="B218" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="B219" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="B220" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="B221" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="B222" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="B223" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="B224" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="B225" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="B226" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="B227" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="B228" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="B229" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="B230" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="B231" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="B232" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="B233" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="B234" t="s">
-        <v>237</v>
+        <v>445</v>
       </c>
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
-        <v>451</v>
+        <v>446</v>
       </c>
       <c r="B235" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B236" t="s">
-        <v>450</v>
+        <v>237</v>
       </c>
     </row>
     <row r="237" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="B237" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
     </row>
     <row r="238" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
-        <v>460</v>
+        <v>449</v>
       </c>
       <c r="B238" t="s">
-        <v>461</v>
+        <v>450</v>
       </c>
     </row>
     <row r="239" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
-        <v>462</v>
+        <v>453</v>
       </c>
       <c r="B239" t="s">
-        <v>463</v>
+        <v>454</v>
       </c>
     </row>
     <row r="240" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
       <c r="B240" t="s">
-        <v>47</v>
+        <v>461</v>
       </c>
     </row>
     <row r="241" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
       <c r="B241" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
     </row>
     <row r="242" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="B242" t="s">
-        <v>459</v>
+        <v>47</v>
       </c>
     </row>
     <row r="243" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
-        <v>464</v>
+        <v>456</v>
       </c>
       <c r="B243" t="s">
-        <v>465</v>
+        <v>457</v>
       </c>
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
-        <v>466</v>
+        <v>458</v>
       </c>
       <c r="B244" t="s">
-        <v>467</v>
+        <v>459</v>
       </c>
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="B245" t="s">
-        <v>273</v>
+        <v>465</v>
       </c>
     </row>
     <row r="246" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="B246" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
     </row>
     <row r="247" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="B247" t="s">
-        <v>472</v>
+        <v>273</v>
       </c>
     </row>
     <row r="248" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="B248" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="B249" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="B250" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="B251" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="B252" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
-        <v>483</v>
+        <v>479</v>
       </c>
       <c r="B253" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
     </row>
     <row r="254" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="B254" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
     </row>
     <row r="255" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="B255" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="B256" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="B257" t="s">
-        <v>492</v>
+        <v>488</v>
       </c>
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="B258" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
-        <v>495</v>
+        <v>491</v>
       </c>
       <c r="B259" t="s">
-        <v>496</v>
+        <v>492</v>
       </c>
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A260" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="B260" t="s">
-        <v>498</v>
+        <v>494</v>
       </c>
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A261" t="s">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="B261" t="s">
-        <v>500</v>
+        <v>496</v>
       </c>
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A262" t="s">
-        <v>501</v>
+        <v>497</v>
       </c>
       <c r="B262" t="s">
-        <v>502</v>
+        <v>498</v>
       </c>
     </row>
     <row r="263" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A263" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="B263" t="s">
-        <v>504</v>
+        <v>500</v>
       </c>
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A264" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="B264" t="s">
-        <v>506</v>
+        <v>502</v>
       </c>
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A265" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
       <c r="B265" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A266" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="B266" t="s">
-        <v>510</v>
+        <v>506</v>
       </c>
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A267" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
       <c r="B267" t="s">
-        <v>512</v>
+        <v>508</v>
       </c>
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A268" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="B268" t="s">
-        <v>514</v>
+        <v>510</v>
       </c>
     </row>
     <row r="269" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A269" t="s">
+        <v>511</v>
+      </c>
+      <c r="B269" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A270" t="s">
+        <v>513</v>
+      </c>
+      <c r="B270" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A271" t="s">
         <v>515</v>
       </c>
-      <c r="B269" t="s">
+      <c r="B271" t="s">
         <v>516</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:B1" xr:uid="{57D06625-878C-A840-A829-5EB8C3969019}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B269">
-      <sortCondition ref="A1:A269"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B271">
+      <sortCondition ref="A1:A271"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>